<commit_message>
20250115-1807 add 202412 salemon data.
</commit_message>
<xml_diff>
--- a/Data/EXCEL/Transfer/salemon/202412/1258-salemon-202412.xlsx
+++ b/Data/EXCEL/Transfer/salemon/202412/1258-salemon-202412.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORKSPACES\xls2xlsx\202412\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WORKSPACES\xls2xlsx\Transfer\202412\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35CA73ED-B449-49A6-A3A5-991FBC40D3CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB02F90B-6A6F-4FA3-8BEC-A904790DBF56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{1779BEEA-DDCE-46D6-8500-B63636DDB13F}"/>
+    <workbookView xWindow="2235" yWindow="1695" windowWidth="21600" windowHeight="13425" xr2:uid="{0728EBE0-9BF6-4DE8-A839-A3C08858C87A}"/>
   </bookViews>
   <sheets>
     <sheet name="1258-salemon-202412" sheetId="2" r:id="rId1"/>
@@ -1255,22 +1255,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86466B46-ED42-434D-84C2-7F95BA896F30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{734A0570-87C3-4F95-A648-328FB51767AB}">
   <dimension ref="A1:Q24"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.90625" customWidth="1"/>
-    <col min="2" max="5" width="14.6328125" customWidth="1"/>
-    <col min="6" max="6" width="13.90625" customWidth="1"/>
-    <col min="7" max="7" width="16.08984375" customWidth="1"/>
-    <col min="8" max="10" width="13.90625" customWidth="1"/>
-    <col min="11" max="11" width="14.6328125" customWidth="1"/>
-    <col min="12" max="15" width="13.90625" customWidth="1"/>
-    <col min="16" max="16" width="14.6328125" customWidth="1"/>
-    <col min="17" max="17" width="14.453125" customWidth="1"/>
+    <col min="1" max="1" width="11.875" customWidth="1"/>
+    <col min="2" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="9.5" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="10" width="9.5" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="15" width="9.5" customWidth="1"/>
+    <col min="16" max="16" width="10" customWidth="1"/>
+    <col min="17" max="17" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
@@ -1297,7 +1297,7 @@
       <c r="P1" s="20"/>
       <c r="Q1" s="21"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="17"/>
       <c r="B2" s="16" t="s">
         <v>4</v>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="Q2" s="21"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -1379,7 +1379,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="18"/>
       <c r="B4" s="18"/>
       <c r="C4" s="18"/>
@@ -1418,7 +1418,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>45017</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
         <v>44986</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>44958</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>24.2</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
         <v>44927</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>16.3</v>
       </c>
     </row>
-    <row r="9" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>44896</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
         <v>44866</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>10.9</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>44835</v>
       </c>
@@ -1789,7 +1789,7 @@
         <v>10.1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>44805</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>9.2200000000000006</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>44774</v>
       </c>
@@ -1895,7 +1895,7 @@
         <v>9.52</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>44743</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>8.86</v>
       </c>
     </row>
-    <row r="15" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>44713</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>10.199999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>44682</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>5.62</v>
       </c>
     </row>
-    <row r="17" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>44652</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>5.79</v>
       </c>
     </row>
-    <row r="18" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
         <v>44621</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>5.0199999999999996</v>
       </c>
     </row>
-    <row r="19" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>44593</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>3.37</v>
       </c>
     </row>
-    <row r="20" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>44562</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>13.1</v>
       </c>
     </row>
-    <row r="21" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>44531</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="22" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <v>44501</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>-11.4</v>
       </c>
     </row>
-    <row r="23" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>44470</v>
       </c>
@@ -2425,7 +2425,7 @@
         <v>-13</v>
       </c>
     </row>
-    <row r="24" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>44440</v>
       </c>

</xml_diff>